<commit_message>
test review after 7 days
เทสฟังชั่นการทำงานของระบบเมื่อผู้โดยสารจะรีวิวหลังจาก7วันที่เดินทางในแต่ละครั้ง
</commit_message>
<xml_diff>
--- a/Sprint2/doc/ประวัติการใช้AI.xlsx
+++ b/Sprint2/doc/ประวัติการใช้AI.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\soften\painamnae\Sprint2\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43D0E554-0A87-4415-AF5F-CC01D7D9762C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0D8AB0-42F4-4E58-9F42-58F4DFB11689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ประวัติการใช้ AI" sheetId="3" r:id="rId1"/>
@@ -74,15 +74,6 @@
     <t>ปาณวัฒน์ จันทร์ทองหลาง</t>
   </si>
   <si>
-    <t>Gemini</t>
-  </si>
-  <si>
-    <t>นำปัญญาประดิษฐ์ มาใช้ในขั ้นตอนดังต่อไปนี ้(1) สอบถามปัญหาการdeploy 
-webapp (2) ช่วยในการแก้ปัญหาการdeploy ,databaseบัก ,api 
-google map ไม่แสดง  โดยข้าพเจ้าได้ ตรวจสอบความถูกต้องและแก้ไข
-ข้อผิดพลาดอันเนื่องมาจากผลลัพธ์จากปัญญาประดิษฐ์เรียบร้อยแล้ว</t>
-  </si>
-  <si>
     <t>นางสาวเกษราภรณ์ รุ่งโรจน์มุกดากุล</t>
   </si>
   <si>
@@ -101,6 +92,14 @@
   <si>
     <t>ใช้ในการช่วยแนะนำการทำระบบริวิวและไฟล์.jsต่างๆ</t>
   </si>
+  <si>
+    <t>Gemini ,claude</t>
+  </si>
+  <si>
+    <t>นำปัญญาประดิษฐ์ มาใช้ในขั้นตอนดังต่อไปนี้(1) สอบถามปัญหาการdeploy 
+webapp (2) ช่วยในการแก้ปัญหาการdeploy ,databaseบัก ,api google map ไม่แสดง (3)ช่วยเขียนเทสการรีวิว โดยข้าพเจ้าได้ ตรวจสอบความถูกต้องและแก้ไข
+ข้อผิดพลาดอันเนื่องมาจากผลลัพธ์จากปัญญาประดิษฐ์เรียบร้อยแล้ว</t>
+  </si>
 </sst>
 </file>
 
@@ -117,22 +116,26 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="27"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="20"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -217,9 +220,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
@@ -447,11 +450,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="55.5" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="6"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -651,10 +654,10 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -682,13 +685,13 @@
     </row>
     <row r="8" spans="1:26" ht="77.400000000000006" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -716,13 +719,13 @@
     </row>
     <row r="9" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>

</xml_diff>